<commit_message>
Use Czech-only product descriptions in V-TOP Europe HS summary
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JCyRqyxfsq6EsUgP3FRcST
</commit_message>
<xml_diff>
--- a/output/HS_Code_Summary_V-TOP_Europe_WPXA26B0613CZ456.xlsx
+++ b/output/HS_Code_Summary_V-TOP_Europe_WPXA26B0613CZ456.xlsx
@@ -82,7 +82,7 @@
   <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" wrapText="1"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -471,17 +471,17 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="60" customWidth="1" min="2" max="2"/>
+    <col width="55" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
     <col width="14" customWidth="1" min="7" max="7"/>
     <col width="16" customWidth="1" min="8" max="8"/>
     <col width="55" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="30" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>HS kód</t>
@@ -524,7 +524,7 @@
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>TARIC / poznámka / CBAM / Antidumping</t>
+          <t>Poznámka</t>
         </is>
       </c>
     </row>
@@ -536,7 +536,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>EAS bezpečnostní prvky s magnetickým zámkem – samoobslužné schránky (Alarm Box Wrap), štítky na lahve (Bottle Cap) a tvrdé etikety RF/AM (HD tagy, stop lock, clamp tag) – ochrana zboží proti krádeži v obchodech</t>
+          <t>Pevné samoobslužné schránky a tvrdé etikety (štítky) s magnetickým zámkem, technologie RF/AM – určeno k ochraně zboží proti krádeži v obchodech</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -559,7 +559,7 @@
       <c r="H2" s="2" t="n"/>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>Položky AS1103E, BT3042, HD2036, HD2071, HD2150, HD2045 (6 řádků faktury sloučeno)</t>
+          <t>Sloučeno 6 řádků faktury (kódy AS1103E, BT3042, HD2036, HD2071, HD2150, HD2045)</t>
         </is>
       </c>
     </row>
@@ -571,7 +571,7 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Měkké RF etikety s tištěným obvodem (roll labels 8.2 MHz, deaktivovatelné) – bílé, s čárovým kódem, transparentní</t>
+          <t>Měkké plastové etikety RF s tištěným obvodem, deaktivovatelné, s falešným čárovým kódem – ochrana zboží proti krádeži</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
@@ -594,7 +594,7 @@
       <c r="H3" s="2" t="n"/>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>Položky RL4601, RL4609, RL4719 (3 řádky faktury sloučeny)</t>
+          <t>Sloučeny 3 řádky faktury (kódy RL4601, RL4609, RL4719)</t>
         </is>
       </c>
     </row>
@@ -606,7 +606,7 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>Ocelová/poplastovaná lanka (lanyard, délka 175 mm) k připojení etikety ke zboží</t>
+          <t>Ocelová/poplastovaná lanka sloužící k připojení etikety ke zboží</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
@@ -633,7 +633,7 @@
       </c>
       <c r="I4" s="3" t="inlineStr">
         <is>
-          <t>Kap. 73 – doloženo prohlášení dodavatele o neruském původu oceli (Statement 17.6.2026). AD clo na ocelová lana z CN (ex 7312 10) se na kód 7312 90 00 nevztahuje – ověřit při podání JSD.</t>
+          <t>Kap. 73 – doloženo prohlášení dodavatele o neruském původu oceli (Statement 17.6.2026). Antidumpingové clo na ocelová lana z ČLR se týká jen ex 7312 10 – kód 7312 90 00 mimo rozsah, ověřit při podání JSD.</t>
         </is>
       </c>
     </row>
@@ -645,7 +645,7 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Magnetický oddělovač (uvolňovač) pevných štítků – Dome Detacher DT054</t>
+          <t>Magnetický oddělovač pro pevné štítky (uvolňovač etiket)</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
@@ -668,7 +668,7 @@
       <c r="H5" s="2" t="n"/>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>Dle interní tabulky HS kódů 8505 11 10 – ověřit plný 10místný TARIC při podání</t>
+          <t>Kód DT4013. Dle interní tabulky HS 8505 11 10 – ověřit plný 10místný TARIC při podání.</t>
         </is>
       </c>
     </row>
@@ -680,7 +680,7 @@
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>Bezpečnostní špendlíky pro tvrdé štítky – Dome Plastic Pin, plastová hlava, 16 mm</t>
+          <t>Bezpečnostní špendlíky pro tvrdé štítky (s plastovou hlavou, 16 mm)</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
@@ -707,7 +707,7 @@
       </c>
       <c r="I6" s="3" t="inlineStr">
         <is>
-          <t>Kap. 73 – doloženo prohlášení dodavatele o neruském původu oceli (Statement 17.6.2026)</t>
+          <t>Kap. 73 – doloženo prohlášení dodavatele o neruském původu oceli (Statement 17.6.2026). Kód PN6011.</t>
         </is>
       </c>
     </row>
@@ -802,7 +802,7 @@
       </c>
       <c r="B14" s="8" t="inlineStr">
         <is>
-          <t>Kartonová GW 2815,40 kg + palety 75,00 kg rozpočítány proporcionálně (faktor 1,026638) → celkem 2890,40 kg dle B/L.</t>
+          <t>Kartonová GW 2815,40 kg + palety 75,00 kg rozpočítány proporcionálně (faktor 1,026638) → celkem 2890,40 kg dle B/L. Čisté hmotnosti převzaty přímo z packing listu.</t>
         </is>
       </c>
     </row>
@@ -999,7 +999,7 @@
     <row r="30">
       <c r="A30" s="8" t="inlineStr">
         <is>
-          <t>DT4013 (Dome Detacher): dle interní tabulky 8505 11 10 (magnetický oddělovač, kromě DT4002/DT4052).</t>
+          <t>DT4013 (oddělovač): dle interní tabulky 8505 11 10 (magnetický oddělovač, kromě DT4002/DT4052).</t>
         </is>
       </c>
     </row>
@@ -1013,7 +1013,7 @@
     <row r="32">
       <c r="A32" s="8" t="inlineStr">
         <is>
-          <t>LD3603 se na faktuře vyskytuje 2× (grooved pin / smooth pin) – sloučeno do jednoho HS kódu 7312 90 00 00.</t>
+          <t>LD3603 se na faktuře vyskytuje 2× (drážkovaný / hladký trn) – sloučeno do jednoho HS kódu 7312 90 00 00.</t>
         </is>
       </c>
     </row>

</xml_diff>